<commit_message>
Added initial recording spreadsheets
</commit_message>
<xml_diff>
--- a/probe_data_IV.xlsx
+++ b/probe_data_IV.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="514" uniqueCount="110">
   <si>
     <t xml:space="preserve">rat_ID</t>
   </si>
@@ -41,6 +41,9 @@
   </si>
   <si>
     <t xml:space="preserve">probe_type</t>
+  </si>
+  <si>
+    <t xml:space="preserve">num_channels</t>
   </si>
   <si>
     <t xml:space="preserve">gender</t>
@@ -494,8 +497,8 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:AC92"/>
-  <sheetFormatPr defaultRowHeight="15.75" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:AD92"/>
+  <sheetFormatPr defaultRowHeight="12.8" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12.63"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="20.14"/>
@@ -506,7 +509,7 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1025" min="7" style="0" width="12.63"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="69" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -534,19 +537,22 @@
       <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="3" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="3" t="s">
         <v>10</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>11</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="C2" s="4" t="n">
         <v>26</v>
@@ -555,25 +561,28 @@
         <v>0</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>14</v>
-      </c>
-      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="I2" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="K2" s="4"/>
+      <c r="G2" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J2" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L2" s="4"/>
     </row>
     <row r="3" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="C3" s="4" t="n">
         <v>26</v>
@@ -582,25 +591,28 @@
         <v>0</v>
       </c>
       <c r="E3" s="4" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G3" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I3" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="K3" s="4"/>
-    </row>
-    <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H3" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J3" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="L3" s="4"/>
+    </row>
+    <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C4" s="4" t="n">
         <v>27</v>
@@ -609,21 +621,21 @@
         <v>1</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I4" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>27</v>
@@ -632,21 +644,21 @@
         <v>1</v>
       </c>
       <c r="E5" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I5" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>27</v>
@@ -655,21 +667,21 @@
         <v>1</v>
       </c>
       <c r="E6" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G6" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I6" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J6" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B7" s="4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C7" s="4" t="n">
         <v>27</v>
@@ -678,21 +690,21 @@
         <v>1</v>
       </c>
       <c r="E7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>27</v>
@@ -701,21 +713,21 @@
         <v>1</v>
       </c>
       <c r="E8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>27</v>
@@ -724,21 +736,21 @@
         <v>1</v>
       </c>
       <c r="E9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C10" s="4" t="n">
         <v>27</v>
@@ -747,21 +759,21 @@
         <v>1</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I10" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B11" s="4" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C11" s="4" t="n">
         <v>27</v>
@@ -770,18 +782,18 @@
         <v>1</v>
       </c>
       <c r="E11" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G11" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I11" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>21</v>
+      </c>
+      <c r="H11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" s="4" t="n">
         <v>28</v>
@@ -790,18 +802,21 @@
         <v>1</v>
       </c>
       <c r="E12" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G12" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="C13" s="4" t="n">
         <v>31</v>
@@ -810,21 +825,24 @@
         <v>0</v>
       </c>
       <c r="E13" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F13" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G13" s="4" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G13" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C14" s="4" t="n">
         <v>27</v>
@@ -833,27 +851,30 @@
         <v>1</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F14" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G14" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G14" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H14" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J14" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C15" s="4" t="n">
         <v>27</v>
@@ -862,27 +883,30 @@
         <v>1</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F15" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G15" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G15" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H15" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I15" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J15" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B16" s="4" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C16" s="4" t="n">
         <v>27</v>
@@ -891,27 +915,30 @@
         <v>1</v>
       </c>
       <c r="E16" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G16" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G16" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H16" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I16" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J16" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C17" s="4" t="n">
         <v>27</v>
@@ -920,27 +947,30 @@
         <v>1</v>
       </c>
       <c r="E17" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G17" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G17" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H17" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I17" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J17" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C18" s="4" t="n">
         <v>27</v>
@@ -949,27 +979,30 @@
         <v>1</v>
       </c>
       <c r="E18" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F18" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G18" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G18" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H18" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I18" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J18" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C19" s="4" t="n">
         <v>27</v>
@@ -978,27 +1011,30 @@
         <v>1</v>
       </c>
       <c r="E19" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F19" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G19" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G19" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H19" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I19" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J19" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C20" s="4" t="n">
         <v>27</v>
@@ -1007,27 +1043,30 @@
         <v>1</v>
       </c>
       <c r="E20" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F20" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G20" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G20" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H20" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I20" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J20" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C21" s="4" t="n">
         <v>27</v>
@@ -1036,24 +1075,27 @@
         <v>1</v>
       </c>
       <c r="E21" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F21" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G21" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G21" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H21" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I21" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J21" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C22" s="4" t="n">
         <v>30</v>
@@ -1062,27 +1104,30 @@
         <v>0</v>
       </c>
       <c r="E22" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="G22" s="4" t="s">
-        <v>34</v>
+        <v>44</v>
+      </c>
+      <c r="G22" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H22" s="4" t="s">
         <v>35</v>
       </c>
       <c r="I22" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>36</v>
+      </c>
+      <c r="J22" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="C23" s="4" t="n">
         <v>20</v>
@@ -1091,21 +1136,24 @@
         <v>1</v>
       </c>
       <c r="E23" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F23" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G23" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G23" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H23" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="C24" s="4" t="n">
         <v>20</v>
@@ -1114,21 +1162,24 @@
         <v>1</v>
       </c>
       <c r="E24" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F24" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G24" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G24" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H24" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C25" s="4" t="n">
         <v>20</v>
@@ -1137,21 +1188,24 @@
         <v>1</v>
       </c>
       <c r="E25" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F25" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G25" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G25" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H25" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C26" s="4" t="n">
         <v>20</v>
@@ -1160,21 +1214,24 @@
         <v>1</v>
       </c>
       <c r="E26" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F26" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G26" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G26" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H26" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="C27" s="4" t="n">
         <v>20</v>
@@ -1183,21 +1240,24 @@
         <v>1</v>
       </c>
       <c r="E27" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F27" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G27" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G27" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H27" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C28" s="4" t="n">
         <v>20</v>
@@ -1206,21 +1266,24 @@
         <v>1</v>
       </c>
       <c r="E28" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F28" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G28" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G28" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H28" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="C29" s="4" t="n">
         <v>20</v>
@@ -1229,21 +1292,24 @@
         <v>1</v>
       </c>
       <c r="E29" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F29" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G29" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G29" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H29" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="4" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C30" s="4" t="n">
         <v>20</v>
@@ -1252,21 +1318,24 @@
         <v>1</v>
       </c>
       <c r="E30" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F30" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G30" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G30" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H30" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C31" s="4" t="n">
         <v>23</v>
@@ -1275,24 +1344,27 @@
         <v>1</v>
       </c>
       <c r="E31" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F31" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G31" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I31" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G31" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H31" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J31" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C32" s="4" t="n">
         <v>23</v>
@@ -1301,24 +1373,27 @@
         <v>1</v>
       </c>
       <c r="E32" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F32" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I32" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G32" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H32" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J32" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C33" s="4" t="n">
         <v>23</v>
@@ -1327,24 +1402,27 @@
         <v>1</v>
       </c>
       <c r="E33" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F33" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G33" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I33" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G33" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H33" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J33" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C34" s="4" t="n">
         <v>23</v>
@@ -1353,24 +1431,27 @@
         <v>1</v>
       </c>
       <c r="E34" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F34" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G34" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I34" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G34" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H34" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J34" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="C35" s="4" t="n">
         <v>23</v>
@@ -1379,24 +1460,27 @@
         <v>1</v>
       </c>
       <c r="E35" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F35" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G35" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I35" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G35" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H35" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J35" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C36" s="4" t="n">
         <v>23</v>
@@ -1405,24 +1489,27 @@
         <v>1</v>
       </c>
       <c r="E36" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F36" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G36" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I36" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G36" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H36" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J36" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="C37" s="4" t="n">
         <v>23</v>
@@ -1431,21 +1518,24 @@
         <v>1</v>
       </c>
       <c r="E37" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F37" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G37" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I37" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>19</v>
+      </c>
+      <c r="G37" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H37" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J37" s="4" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C38" s="4" t="n">
         <v>25</v>
@@ -1454,21 +1544,24 @@
         <v>1</v>
       </c>
       <c r="E38" s="4" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F38" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G38" s="4" t="s">
-        <v>15</v>
+        <v>19</v>
+      </c>
+      <c r="G38" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H38" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I38" s="4" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="C39" s="4" t="n">
         <v>24</v>
@@ -1477,21 +1570,24 @@
         <v>1</v>
       </c>
       <c r="E39" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F39" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="G39" s="4" t="s">
-        <v>34</v>
+        <v>19</v>
+      </c>
+      <c r="G39" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H39" s="4" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="I39" s="4" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="C40" s="4" t="n">
         <v>31</v>
@@ -1500,19 +1596,22 @@
         <v>1</v>
       </c>
       <c r="E40" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="F40" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G40" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H40" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="F40" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G40" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="4" t="s">
-        <v>65</v>
-      </c>
       <c r="C41" s="4" t="n">
         <v>32</v>
       </c>
@@ -1520,21 +1619,24 @@
         <v>1</v>
       </c>
       <c r="E41" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F41" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G41" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G41" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H41" s="4" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="I41" s="4" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="C42" s="4" t="n">
         <v>25</v>
@@ -1543,18 +1645,21 @@
         <v>1</v>
       </c>
       <c r="E42" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F42" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G42" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H42" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="F42" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G42" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="C43" s="4" t="n">
         <v>26</v>
@@ -1563,18 +1668,21 @@
         <v>2</v>
       </c>
       <c r="E43" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F43" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G43" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H43" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="F43" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G43" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="C44" s="4" t="n">
         <v>27</v>
@@ -1583,21 +1691,24 @@
         <v>1</v>
       </c>
       <c r="E44" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F44" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G44" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H44" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I44" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="F44" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G44" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H44" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="C45" s="4" t="n">
         <v>29</v>
@@ -1606,21 +1717,24 @@
         <v>1</v>
       </c>
       <c r="E45" s="4" t="s">
+        <v>70</v>
+      </c>
+      <c r="F45" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G45" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H45" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I45" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="F45" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G45" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H45" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="4" t="s">
-        <v>68</v>
       </c>
       <c r="C46" s="4" t="n">
         <v>29</v>
@@ -1629,21 +1743,24 @@
         <v>2</v>
       </c>
       <c r="E46" s="4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="F46" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G46" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G46" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H46" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="I46" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C47" s="4" t="n">
         <v>26</v>
@@ -1652,18 +1769,21 @@
         <v>1</v>
       </c>
       <c r="E47" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F47" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G47" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G47" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H47" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C48" s="4" t="n">
         <v>27</v>
@@ -1672,21 +1792,24 @@
         <v>1</v>
       </c>
       <c r="E48" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F48" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G48" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G48" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H48" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="I48" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C49" s="4" t="n">
         <v>27</v>
@@ -1695,18 +1818,21 @@
         <v>2</v>
       </c>
       <c r="E49" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F49" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G49" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G49" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H49" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="C50" s="4" t="n">
         <v>29</v>
@@ -1715,24 +1841,27 @@
         <v>2</v>
       </c>
       <c r="E50" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="F50" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G50" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G50" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H50" s="4" t="s">
-        <v>71</v>
+        <v>35</v>
+      </c>
+      <c r="I50" s="4" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="C51" s="4" t="n">
         <v>17</v>
@@ -1741,68 +1870,74 @@
         <v>1</v>
       </c>
       <c r="E51" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F51" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G51" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G51" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H51" s="4" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I51" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J51" s="0" t="s">
-        <v>16</v>
+        <v>77</v>
+      </c>
+      <c r="J51" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="K51" s="0" t="s">
-        <v>77</v>
+        <v>17</v>
+      </c>
+      <c r="L51" s="0" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B52" s="4" t="s">
+        <v>79</v>
+      </c>
+      <c r="C52" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="D52" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="4" t="s">
+        <v>76</v>
+      </c>
+      <c r="F52" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G52" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H52" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I52" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="J52" s="4" t="s">
+        <v>17</v>
+      </c>
+      <c r="K52" s="0" t="s">
+        <v>17</v>
+      </c>
+      <c r="L52" s="0" t="s">
         <v>78</v>
-      </c>
-      <c r="C52" s="4" t="n">
-        <v>17</v>
-      </c>
-      <c r="D52" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E52" s="4" t="s">
-        <v>75</v>
-      </c>
-      <c r="F52" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G52" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H52" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="I52" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J52" s="0" t="s">
-        <v>16</v>
-      </c>
-      <c r="K52" s="0" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C53" s="4" t="n">
         <v>17</v>
@@ -1811,33 +1946,36 @@
         <v>1</v>
       </c>
       <c r="E53" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F53" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G53" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G53" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H53" s="4" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I53" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J53" s="0" t="s">
-        <v>16</v>
+        <v>77</v>
+      </c>
+      <c r="J53" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="K53" s="0" t="s">
-        <v>77</v>
+        <v>17</v>
+      </c>
+      <c r="L53" s="0" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="54" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A54" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B54" s="4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="C54" s="4" t="n">
         <v>17</v>
@@ -1846,33 +1984,36 @@
         <v>1</v>
       </c>
       <c r="E54" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F54" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G54" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G54" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H54" s="4" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I54" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J54" s="0" t="s">
-        <v>16</v>
+        <v>77</v>
+      </c>
+      <c r="J54" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="K54" s="0" t="s">
-        <v>77</v>
+        <v>17</v>
+      </c>
+      <c r="L54" s="0" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="55" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B55" s="4" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C55" s="4" t="n">
         <v>17</v>
@@ -1881,33 +2022,36 @@
         <v>1</v>
       </c>
       <c r="E55" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F55" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G55" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G55" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H55" s="4" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I55" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J55" s="0" t="s">
-        <v>16</v>
+        <v>77</v>
+      </c>
+      <c r="J55" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="K55" s="0" t="s">
-        <v>77</v>
+        <v>17</v>
+      </c>
+      <c r="L55" s="0" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B56" s="4" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C56" s="4" t="n">
         <v>17</v>
@@ -1916,33 +2060,36 @@
         <v>1</v>
       </c>
       <c r="E56" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F56" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G56" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G56" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H56" s="4" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I56" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J56" s="0" t="s">
-        <v>16</v>
+        <v>77</v>
+      </c>
+      <c r="J56" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="K56" s="0" t="s">
-        <v>77</v>
+        <v>17</v>
+      </c>
+      <c r="L56" s="0" t="s">
+        <v>78</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A57" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B57" s="4" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C57" s="4" t="n">
         <v>17</v>
@@ -1951,30 +2098,33 @@
         <v>1</v>
       </c>
       <c r="E57" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F57" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G57" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G57" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H57" s="4" t="s">
-        <v>76</v>
+        <v>16</v>
       </c>
       <c r="I57" s="4" t="s">
-        <v>16</v>
-      </c>
-      <c r="J57" s="0" t="s">
-        <v>16</v>
+        <v>77</v>
+      </c>
+      <c r="J57" s="4" t="s">
+        <v>17</v>
       </c>
       <c r="K57" s="0" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="58" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>17</v>
+      </c>
+      <c r="L57" s="0" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C58" s="4" t="n">
         <v>18</v>
@@ -1983,24 +2133,27 @@
         <v>2</v>
       </c>
       <c r="E58" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F58" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G58" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G58" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H58" s="4" t="s">
-        <v>84</v>
+        <v>16</v>
+      </c>
+      <c r="I58" s="4" t="s">
+        <v>85</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B59" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C59" s="4" t="n">
         <v>19</v>
@@ -2009,24 +2162,27 @@
         <v>1</v>
       </c>
       <c r="E59" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F59" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G59" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G59" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H59" s="4" t="s">
-        <v>70</v>
+        <v>16</v>
+      </c>
+      <c r="I59" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B60" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C60" s="4" t="n">
         <v>19</v>
@@ -2035,24 +2191,27 @@
         <v>1</v>
       </c>
       <c r="E60" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F60" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G60" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G60" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H60" s="4" t="s">
-        <v>70</v>
+        <v>16</v>
+      </c>
+      <c r="I60" s="4" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="61" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B61" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C61" s="4" t="n">
         <v>19</v>
@@ -2061,24 +2220,27 @@
         <v>1</v>
       </c>
       <c r="E61" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F61" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G61" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G61" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H61" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="62" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I61" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="62" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A62" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B62" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C62" s="4" t="n">
         <v>19</v>
@@ -2087,24 +2249,27 @@
         <v>1</v>
       </c>
       <c r="E62" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F62" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G62" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G62" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H62" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="63" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I62" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="63" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B63" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C63" s="4" t="n">
         <v>19</v>
@@ -2113,24 +2278,27 @@
         <v>1</v>
       </c>
       <c r="E63" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F63" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G63" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G63" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H63" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="64" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I63" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="64" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B64" s="4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="C64" s="4" t="n">
         <v>19</v>
@@ -2139,24 +2307,27 @@
         <v>1</v>
       </c>
       <c r="E64" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F64" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G64" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G64" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H64" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="65" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I64" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="65" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B65" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="C65" s="4" t="n">
         <v>19</v>
@@ -2165,21 +2336,24 @@
         <v>1</v>
       </c>
       <c r="E65" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F65" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G65" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G65" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H65" s="4" t="s">
-        <v>70</v>
-      </c>
-    </row>
-    <row r="66" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I65" s="4" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="66" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C66" s="4" t="n">
         <v>20</v>
@@ -2188,21 +2362,24 @@
         <v>2</v>
       </c>
       <c r="E66" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F66" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G66" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G66" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H66" s="4" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="67" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I66" s="4" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A67" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C67" s="4" t="n">
         <v>21</v>
@@ -2211,21 +2388,24 @@
         <v>0</v>
       </c>
       <c r="E67" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F67" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G67" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G67" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H67" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="68" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I67" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A68" s="4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C68" s="4" t="n">
         <v>22</v>
@@ -2234,21 +2414,24 @@
         <v>0</v>
       </c>
       <c r="E68" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F68" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G68" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G68" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H68" s="4" t="s">
-        <v>92</v>
-      </c>
-    </row>
-    <row r="69" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I68" s="4" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A69" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C69" s="4" t="n">
         <v>17</v>
@@ -2257,21 +2440,24 @@
         <v>0</v>
       </c>
       <c r="E69" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F69" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G69" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G69" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H69" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="70" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="I69" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A70" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C70" s="4" t="n">
         <v>16</v>
@@ -2280,44 +2466,50 @@
         <v>0</v>
       </c>
       <c r="E70" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F70" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G70" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H70" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I70" s="4" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A71" s="4" t="s">
+        <v>95</v>
+      </c>
+      <c r="C71" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="D71" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="E71" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="G70" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H70" s="4" t="s">
+      <c r="F71" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G71" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H71" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I71" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A72" s="4" t="s">
         <v>95</v>
-      </c>
-    </row>
-    <row r="71" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A71" s="4" t="s">
-        <v>94</v>
-      </c>
-      <c r="C71" s="4" t="n">
-        <v>16</v>
-      </c>
-      <c r="D71" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E71" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F71" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G71" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H71" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="72" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A72" s="4" t="s">
-        <v>94</v>
       </c>
       <c r="C72" s="4" t="n">
         <v>18</v>
@@ -2326,21 +2518,24 @@
         <v>1</v>
       </c>
       <c r="E72" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="F72" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G72" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G72" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H72" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="73" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="I72" s="4" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="73" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A73" s="4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="C73" s="4" t="n">
         <v>19</v>
@@ -2349,21 +2544,24 @@
         <v>2</v>
       </c>
       <c r="E73" s="4" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="F73" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G73" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G73" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H73" s="4" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="74" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>35</v>
+      </c>
+      <c r="I73" s="4" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="74" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A74" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C74" s="4" t="n">
         <v>18</v>
@@ -2372,21 +2570,24 @@
         <v>1</v>
       </c>
       <c r="E74" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F74" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G74" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G74" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H74" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I74" s="4" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A75" s="4" t="s">
         <v>98</v>
-      </c>
-    </row>
-    <row r="75" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A75" s="4" t="s">
-        <v>97</v>
       </c>
       <c r="C75" s="4" t="n">
         <v>20</v>
@@ -2395,21 +2596,24 @@
         <v>1</v>
       </c>
       <c r="E75" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F75" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G75" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G75" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H75" s="4" t="s">
-        <v>99</v>
-      </c>
-    </row>
-    <row r="76" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I75" s="4" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="76" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A76" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C76" s="4" t="n">
         <v>22</v>
@@ -2418,21 +2622,24 @@
         <v>1</v>
       </c>
       <c r="E76" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F76" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G76" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G76" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H76" s="4" t="s">
-        <v>101</v>
-      </c>
-    </row>
-    <row r="77" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I76" s="4" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="77" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A77" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="C77" s="4" t="n">
         <v>23</v>
@@ -2441,21 +2648,24 @@
         <v>2</v>
       </c>
       <c r="E77" s="4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="F77" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G77" s="4" t="s">
-        <v>15</v>
+        <v>34</v>
+      </c>
+      <c r="G77" s="4" t="n">
+        <v>32</v>
       </c>
       <c r="H77" s="4" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="78" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>16</v>
+      </c>
+      <c r="I77" s="4" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="78" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A78" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="C78" s="4" t="n">
         <v>17</v>
@@ -2464,21 +2674,24 @@
         <v>1</v>
       </c>
       <c r="E78" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F78" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G78" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I78" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G78" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H78" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J78" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="79" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A79" s="4" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="79" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A79" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="C79" s="4" t="n">
         <v>18</v>
@@ -2487,21 +2700,24 @@
         <v>1</v>
       </c>
       <c r="E79" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F79" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G79" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="I79" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G79" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H79" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="J79" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="80" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A80" s="4" t="s">
         <v>104</v>
-      </c>
-    </row>
-    <row r="80" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A80" s="4" t="s">
-        <v>103</v>
       </c>
       <c r="B80" s="4"/>
       <c r="C80" s="4" t="n">
@@ -2511,19 +2727,21 @@
         <v>1</v>
       </c>
       <c r="E80" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F80" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G80" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="H80" s="4"/>
-      <c r="I80" s="4" t="s">
-        <v>104</v>
-      </c>
-      <c r="J80" s="4"/>
+        <v>34</v>
+      </c>
+      <c r="G80" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H80" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="I80" s="4"/>
+      <c r="J80" s="4" t="s">
+        <v>105</v>
+      </c>
       <c r="K80" s="4"/>
       <c r="L80" s="4"/>
       <c r="M80" s="4"/>
@@ -2543,10 +2761,11 @@
       <c r="AA80" s="4"/>
       <c r="AB80" s="4"/>
       <c r="AC80" s="4"/>
-    </row>
-    <row r="81" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="AD80" s="4"/>
+    </row>
+    <row r="81" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A81" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C81" s="4" t="n">
         <v>18</v>
@@ -2555,21 +2774,24 @@
         <v>1</v>
       </c>
       <c r="E81" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F81" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G81" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I81" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="82" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G81" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H81" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J81" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="82" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A82" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="C82" s="4" t="n">
         <v>19</v>
@@ -2578,21 +2800,24 @@
         <v>1</v>
       </c>
       <c r="E82" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F82" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G82" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="I82" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="83" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G82" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H82" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="J82" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="83" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A83" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B83" s="4"/>
       <c r="C83" s="4" t="n">
@@ -2602,22 +2827,25 @@
         <v>1</v>
       </c>
       <c r="E83" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F83" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G83" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H83" s="4"/>
-      <c r="I83" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="84" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G83" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H83" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I83" s="4"/>
+      <c r="J83" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="84" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A84" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B84" s="4"/>
       <c r="C84" s="4" t="n">
@@ -2627,22 +2855,25 @@
         <v>2</v>
       </c>
       <c r="E84" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F84" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G84" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H84" s="4"/>
-      <c r="I84" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="85" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G84" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H84" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I84" s="4"/>
+      <c r="J84" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="85" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A85" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B85" s="4"/>
       <c r="C85" s="4" t="n">
@@ -2652,22 +2883,25 @@
         <v>1</v>
       </c>
       <c r="E85" s="4" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F85" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G85" s="4" t="s">
-        <v>34</v>
-      </c>
-      <c r="H85" s="4"/>
-      <c r="I85" s="4" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="86" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G85" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H85" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="I85" s="4"/>
+      <c r="J85" s="4" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="86" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A86" s="4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="C86" s="4" t="n">
         <v>17</v>
@@ -2676,18 +2910,21 @@
         <v>1</v>
       </c>
       <c r="E86" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F86" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G86" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H86" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="87" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A87" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="F86" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G86" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="87" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A87" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="C87" s="4" t="n">
         <v>19</v>
@@ -2696,18 +2933,21 @@
         <v>1</v>
       </c>
       <c r="E87" s="4" t="s">
+        <v>108</v>
+      </c>
+      <c r="F87" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="G87" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H87" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="88" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A88" s="4" t="s">
         <v>107</v>
-      </c>
-      <c r="F87" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G87" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="88" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A88" s="4" t="s">
-        <v>106</v>
       </c>
       <c r="C88" s="4" t="n">
         <v>23</v>
@@ -2716,18 +2956,21 @@
         <v>1</v>
       </c>
       <c r="E88" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F88" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G88" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="89" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G88" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H88" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="89" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A89" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C89" s="4" t="n">
         <v>18</v>
@@ -2736,18 +2979,21 @@
         <v>1</v>
       </c>
       <c r="E89" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F89" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G89" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="90" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G89" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H89" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="90" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A90" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C90" s="4" t="n">
         <v>21</v>
@@ -2756,18 +3002,21 @@
         <v>2</v>
       </c>
       <c r="E90" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F90" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G90" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="91" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G90" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H90" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="91" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A91" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C91" s="4" t="n">
         <v>22</v>
@@ -2776,18 +3025,21 @@
         <v>1</v>
       </c>
       <c r="E91" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F91" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G91" s="4" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="92" customFormat="false" ht="15.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+      <c r="G91" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H91" s="4" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="92" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A92" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="C92" s="4" t="n">
         <v>24</v>
@@ -2796,13 +3048,16 @@
         <v>1</v>
       </c>
       <c r="E92" s="4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="F92" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G92" s="4" t="s">
-        <v>34</v>
+        <v>34</v>
+      </c>
+      <c r="G92" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="H92" s="4" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>